<commit_message>
5 exchange tests finished
</commit_message>
<xml_diff>
--- a/NineMdRobot/Test_Cases.xlsx
+++ b/NineMdRobot/Test_Cases.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\Python\QA_Testing\NineMdRobot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31958D95-EA76-491B-8A32-A2C33B5C5795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C49934D9-C384-4EFB-BE52-79727CE6AEEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{652417F1-FFEB-4421-A0A4-47EF781B78EA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{652417F1-FFEB-4421-A0A4-47EF781B78EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet name="Problems Found" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="67">
   <si>
     <t>ID</t>
   </si>
@@ -79,9 +80,6 @@
   </si>
   <si>
     <t>Input fields accept numbers</t>
-  </si>
-  <si>
-    <t>Input fields reject keys that are not numbers</t>
   </si>
   <si>
     <t>1. Input field is highlighted
@@ -93,24 +91,10 @@
     <t>TC_InputValues_004</t>
   </si>
   <si>
-    <t>1. Input field is highlighted
-2. All fields show '0'
-3.1 MDL Input field has '123.9' value
-3.2. All currencies change dynamically to be different than '0'</t>
-  </si>
-  <si>
     <t>Changing the Bank updates the Currencies</t>
   </si>
   <si>
-    <t>Editing a new field updates all other fields</t>
-  </si>
-  <si>
     <t>Currency exchange is calculated correctly</t>
-  </si>
-  <si>
-    <t>1. Click the MDL input field
-2. Delete default value
-3. Type '123.9'</t>
   </si>
   <si>
     <t>1. Click the MDL input field
@@ -127,11 +111,6 @@
   </si>
   <si>
     <t>TC_Exchange_001</t>
-  </si>
-  <si>
-    <t>1. Click the Main dropdown button
-2. Click the Bank dropdown button
-3. Pick 'Energbank'</t>
   </si>
   <si>
     <t>1. More currencies appear
@@ -232,10 +211,79 @@
 6. Type '456'</t>
   </si>
   <si>
-    <t>Done</t>
-  </si>
-  <si>
-    <t>State</t>
+    <t>Input fields ignore keys that are not numbers</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>API currency rates needed for test automation</t>
+  </si>
+  <si>
+    <t>1. Click any input field
+2. Delete default value
+3. Type '123.9'</t>
+  </si>
+  <si>
+    <t>1. Input field is highlighted
+2. All fields show '0'
+3.1 Edited Input field has '123.9' value
+3.2. All currencies change dynamically to be different than '0'</t>
+  </si>
+  <si>
+    <t>TC_Exchange_002</t>
+  </si>
+  <si>
+    <t>Currency exchange works when bank is changed</t>
+  </si>
+  <si>
+    <t>1. Click the Main dropdown button
+2. Click the Bank dropdown button
+3. Pick any bank from list
+4. Type '1' in any currency field</t>
+  </si>
+  <si>
+    <t>Editing a new field updates all other fields in extended currency view</t>
+  </si>
+  <si>
+    <t>I am on the home page
+Currency dropdown button clicked</t>
+  </si>
+  <si>
+    <t>1. Click the Currency dropdown button
+2. Click the Bank dropdown button
+3. Pick 'Energbank'</t>
+  </si>
+  <si>
+    <t>I am on the home page
+Currency API is functional</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Environment Details</t>
+  </si>
+  <si>
+    <t>Steps to Reproduce</t>
+  </si>
+  <si>
+    <t>Expected vs. Actual Result</t>
+  </si>
+  <si>
+    <t>Browser: Chrome, OS: Windows 11, Automation Tool: Robot Framework + SeleniumLibrary</t>
+  </si>
+  <si>
+    <t>1. Navigate to https://999.md/ro
+2. On currency exchange dialog, press any input field
+3. Press different digits into input field</t>
+  </si>
+  <si>
+    <t>Expected: A limit of 20 digits on input
+Actual: No limit on the digits pressed</t>
+  </si>
+  <si>
+    <t>No limit on number of digits pressed into currency input field</t>
   </si>
 </sst>
 </file>
@@ -619,18 +667,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{241472C1-831D-4A75-B8C7-109A4385B52E}">
-  <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.109375" customWidth="1"/>
-    <col min="2" max="2" width="21.33203125" customWidth="1"/>
-    <col min="3" max="3" width="25.21875" customWidth="1"/>
-    <col min="4" max="4" width="42.88671875" customWidth="1"/>
-    <col min="5" max="5" width="32.21875" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+    <col min="3" max="3" width="25.28515625" customWidth="1"/>
+    <col min="4" max="4" width="42.85546875" customWidth="1"/>
+    <col min="5" max="5" width="32.28515625" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -653,13 +702,13 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -670,51 +719,49 @@
         <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F3">
         <v>2</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -725,199 +772,285 @@
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F4">
         <v>2</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="F5">
         <v>2</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" t="s">
-        <v>10</v>
+        <v>55</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>56</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F7">
         <v>2</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
+        <v>16</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>58</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F8">
         <v>1</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>38</v>
+        <v>53</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>42</v>
+      <c r="D10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="F10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="C11" t="s">
         <v>10</v>
       </c>
+      <c r="D11" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="E11" s="1" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12">
         <v>2</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>43</v>
+      <c r="G12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58F60173-195C-44F3-B687-05744D1943A3}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="55.7109375" customWidth="1"/>
+    <col min="2" max="2" width="79.7109375" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" customWidth="1"/>
+    <col min="5" max="5" width="8.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>